<commit_message>
QLDA: fix import/export Excel đề xuất chuyển tiếp — thêm cột Năm (NamDeXuat)
Đọc và validate NamDeXuat từ Excel thay vì hardcode DateTime.Now.Year.
Đồng bộ template import/export 7 cột và giữ Excel Table DeXuatChuyenTiepImport.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/PrintTemplates/DanhSachDeXuatChuTruongChuyenTiep.xlsx
+++ b/QLDA.WebApi/PrintTemplates/DanhSachDeXuatChuTruongChuyenTiep.xlsx
@@ -1,142 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\PrintTemplates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACD2B35-D9CD-4A11-AC59-7D93C4E2D959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="KetQuaPhanKhaiVon" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KetQuaPhanKhaiVon" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>STT</t>
-  </si>
-  <si>
-    <t>$Stt</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-TRUNG TÂM CHUYỂN ĐỔI SỐ </t>
-    </r>
-  </si>
-  <si>
-    <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
-Độc lập - Tự do - Hạnh phúc
----------------</t>
-  </si>
-  <si>
-    <t>ĐỀ XUẤT CHỦ TRƯƠNG CHUYỂN TIẾP</t>
-  </si>
-  <si>
-    <t>Số liệu giải ngân</t>
-  </si>
-  <si>
-    <t>$SoLieuGiaiNgan</t>
-  </si>
-  <si>
-    <t>ước giải ngân</t>
-  </si>
-  <si>
-    <t>$UocGiaiNgan</t>
-  </si>
-  <si>
-    <t>Nhu cầu kinh phí</t>
-  </si>
-  <si>
-    <t>Khối Lượng đa hoàn thành</t>
-  </si>
-  <si>
-    <t>Khối lượng dự kiến đã hoàn thành</t>
-  </si>
-  <si>
-    <t>$NhuCauKinhPhi</t>
-  </si>
-  <si>
-    <t>$KhoiLuongThucTe</t>
-  </si>
-  <si>
-    <t>$KhoiLuongDuKien</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="6">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="18"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -183,52 +107,112 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -516,105 +500,142 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="22" style="2" customWidth="1"/>
-    <col min="3" max="3" width="40.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="33.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="33.5546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="35.5546875" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="2"/>
+    <col width="7.6640625" customWidth="1" style="2" min="1" max="1"/>
+    <col width="22" customWidth="1" style="2" min="2" max="2"/>
+    <col width="40.44140625" customWidth="1" style="2" min="3" max="3"/>
+    <col width="33.6640625" customWidth="1" style="2" min="4" max="4"/>
+    <col width="33.5546875" customWidth="1" style="2" min="5" max="5"/>
+    <col width="35.5546875" customWidth="1" style="2" min="6" max="6"/>
+    <col width="8.88671875" customWidth="1" style="2" min="7" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="11"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
+TRUNG TÂM CHUYỂN ĐỔI SỐ </t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
+Độc lập - Tự do - Hạnh phúc
+---------------</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="n"/>
+      <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="n"/>
     </row>
-    <row r="2" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
+    <row r="2" ht="13.2" customHeight="1">
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
     </row>
-    <row r="3" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+    <row r="3" ht="22.8" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT CHỦ TRƯƠNG CHUYỂN TIẾP</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="13" t="n"/>
+      <c r="G3" s="13" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>11</v>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Năm</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Số liệu giải ngân</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>ước giải ngân</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Nhu cầu kinh phí</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Khối Lượng đa hoàn thành</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Khối lượng dự kiến đã hoàn thành</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>14</v>
+    <row r="5" ht="14.4" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>$Stt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$NamDeXuat</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>$SoLieuGiaiNgan</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>$UocGiaiNgan</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>$NhuCauKinhPhi</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>$KhoiLuongThucTe</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>$KhoiLuongDuKien</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="E1:F2"/>
-    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>